<commit_message>
Script adaptado de Excel completo con correcciones de valores de dias totales para los bloques
</commit_message>
<xml_diff>
--- a/depredacion_ping.xlsx
+++ b/depredacion_ping.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Análisis_R\Pinguinos\pingML\pinguinosML_2026\Planillas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Análisis_R\Pinguinos\pingML\pinguinosML_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0A04F21-CF40-498C-B2EE-769B8426F4BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C14E6A23-A0AF-4BEE-A5C5-B7BB89AC837F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="480" windowWidth="20730" windowHeight="11160" xr2:uid="{882FD2A0-B437-4AB7-A290-6C9354C7DE59}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{882FD2A0-B437-4AB7-A290-6C9354C7DE59}"/>
   </bookViews>
   <sheets>
     <sheet name="db LIMPIA" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'db LIMPIA'!$A$617:$F$639</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'db LIMPIA'!$G$1:$G$1938</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -13255,7 +13255,7 @@
         <v>7</v>
       </c>
       <c r="F544" s="12">
-        <v>43510</v>
+        <v>42780</v>
       </c>
       <c r="G544" s="13">
         <v>8</v>
@@ -13278,7 +13278,7 @@
         <v>7</v>
       </c>
       <c r="F545" s="12">
-        <v>43510</v>
+        <v>42780</v>
       </c>
       <c r="G545" s="13">
         <v>8</v>
@@ -15901,7 +15901,7 @@
         <v>2</v>
       </c>
       <c r="F659" s="12">
-        <v>45271</v>
+        <v>43080</v>
       </c>
       <c r="G659" s="13">
         <v>4</v>
@@ -15970,7 +15970,7 @@
         <v>3</v>
       </c>
       <c r="F662" s="35">
-        <v>45285</v>
+        <v>43094</v>
       </c>
       <c r="G662" s="13">
         <v>5</v>
@@ -45405,6 +45405,7 @@
       <c r="I1938" s="37"/>
     </row>
   </sheetData>
+  <autoFilter ref="G1:G1938" xr:uid="{2E974311-F8C1-4509-BFA4-E5734A9CD811}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>